<commit_message>
Add handoff doc and requirements.txt for Nitya's environment setup
NITYA_HANDOFF.md orients a fresh Claude session on this repo: what's
relevant (Dezi Art Prize folder) vs. unrelated (the Opportunities Hub
scraper files at repo root), data model, environment setup, the
scraping + email-discovery workflow, the two-branch push routine, and
current project state. requirements.txt pins the exact package
versions used in .venv_crawl4ai (gitignored, must be recreated).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_no_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_no_email.xlsx
@@ -26893,7 +26893,7 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BFA/BA Fine Art (C33 Gallery)</t>
+          <t>BFA Fine Art (C33 Gallery)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -26903,7 +26903,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+          <t>https://www.creatingbyjenna.art/</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -26919,7 +26919,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+          <t>Personal site found via web search (creatingbyjenna.art) but no email visible — only Instagram/TikTok/YouTube and an unfetched /contact page; no email found</t>
         </is>
       </c>
     </row>
@@ -27010,7 +27010,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BFA/BA Fine Art (C33 Gallery)</t>
+          <t>BFA Fine Art (C33 Gallery)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -27020,7 +27020,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+          <t>https://shop.colum.edu/lobotomy-by-ana-lara.html</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -27036,7 +27036,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+          <t>Confirmed as a Columbia Fine Arts student via ShopColumbia listing ('Lobotomy' by Ana Lara) but no email found — ShopColumbia has no direct artist contact page</t>
         </is>
       </c>
     </row>
@@ -27166,7 +27166,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BFA/BA Fine Art (C33 Gallery)</t>
+          <t>BFA Fine Art (C33 Gallery)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -27192,7 +27192,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Name only, from 'C33 Gallery' exhibitor list on the Human Condition 2026 BA/BFA Fine Art Exhibition page; no email/portfolio published</t>
+          <t>No email found — multiple different people share this name online (a Chicago mixed-media artist, a UIC student, a musician endorser); none confirmed as the same Columbia College Chicago student, so not treated as a match</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CalArts Animation scraper: 251 students, 251 with confirmed emails
New source (calarts.edu/filmvideo/animation-student-portfolios/2026/)
covers Character Animation and Experimental Animation across 14
sub-pages (BFA 1-4, Affiliates, Recent Alumni, MFA 1-3). Every student
has a real mailto: link in static HTML -- 100% email yield, the
highest of any source in this project. Kept as a distinct "CalArts
Animation" sheet, separate from the existing names-only "CalArts"
(High Pass) source.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_no_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_no_email.xlsx
@@ -32,6 +32,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iowa" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UW Art" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BGSU" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalArts Animation" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$I$6</definedName>
@@ -59,6 +60,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Iowa'!$A$5:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'UW Art'!$A$5:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'CalArts Animation'!$A$5:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28530,6 +28532,108 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: CalArts Film/Video Animation Student Portfolios, 2026 — Character Animation (BFA 1-4, Affiliates, Recent Alumni) and Experimental Animation (BFA 1-4, MFA 1-3, Recent Alumni), 14 pages total. Each student entry includes name, class year, specialization, and Resume/Email/Portfolio/social links in plain static HTML (no JS rendering needed). Distinct from the separate 'CalArts' source (High Pass BFA exhibition, names only, no email).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://calarts.edu/filmvideo/animation-student-portfolios/2026/character-animation and .../experimental-animation (14 sub-pages: bfa-1 through bfa-4, affiliates, recent-alumni, mfa-1 through mfa-3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>